<commit_message>
Source filter and RC LP OIL update
</commit_message>
<xml_diff>
--- a/VEHAPR26.xlsx
+++ b/VEHAPR26.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5017" uniqueCount="2556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5229" uniqueCount="2558">
   <si>
     <t>NAME</t>
   </si>
@@ -7685,6 +7685,12 @@
   </si>
   <si>
     <t>VIDYADHAR NAGAR</t>
+  </si>
+  <si>
+    <t>WORKSHOP USE</t>
+  </si>
+  <si>
+    <t>TECHNICIAN</t>
   </si>
 </sst>
 </file>
@@ -7720,8 +7726,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8016,12 +8025,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2508"/>
+  <dimension ref="A1:C2614"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="7" customWidth="1"/>
     <col min="6" max="7" width="4" customWidth="1"/>
@@ -35637,6 +35646,1172 @@
         <v>2548</v>
       </c>
     </row>
+    <row r="2509" spans="1:3">
+      <c r="A2509">
+        <v>2508</v>
+      </c>
+      <c r="B2509" s="1" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C2509" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2510" spans="1:3">
+      <c r="A2510">
+        <v>2509</v>
+      </c>
+      <c r="B2510" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="C2510" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2511" spans="1:3">
+      <c r="A2511">
+        <v>2510</v>
+      </c>
+      <c r="B2511" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="C2511" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2512" spans="1:3">
+      <c r="A2512">
+        <v>2511</v>
+      </c>
+      <c r="B2512" s="1" t="s">
+        <v>885</v>
+      </c>
+      <c r="C2512" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2513" spans="1:3">
+      <c r="A2513">
+        <v>2512</v>
+      </c>
+      <c r="B2513" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C2513" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2514" spans="1:3">
+      <c r="A2514">
+        <v>2513</v>
+      </c>
+      <c r="B2514" s="1" t="s">
+        <v>2025</v>
+      </c>
+      <c r="C2514" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2515" spans="1:3">
+      <c r="A2515">
+        <v>2514</v>
+      </c>
+      <c r="B2515" s="1" t="s">
+        <v>639</v>
+      </c>
+      <c r="C2515" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2516" spans="1:3">
+      <c r="A2516">
+        <v>2515</v>
+      </c>
+      <c r="B2516" s="1" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C2516" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2517" spans="1:3">
+      <c r="A2517">
+        <v>2516</v>
+      </c>
+      <c r="B2517" s="1" t="s">
+        <v>1608</v>
+      </c>
+      <c r="C2517" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2518" spans="1:3">
+      <c r="A2518">
+        <v>2517</v>
+      </c>
+      <c r="B2518" s="1" t="s">
+        <v>965</v>
+      </c>
+      <c r="C2518" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2519" spans="1:3">
+      <c r="A2519">
+        <v>2518</v>
+      </c>
+      <c r="B2519" s="1" t="s">
+        <v>1653</v>
+      </c>
+      <c r="C2519" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2520" spans="1:3">
+      <c r="A2520">
+        <v>2519</v>
+      </c>
+      <c r="B2520" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2520" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2521" spans="1:3">
+      <c r="A2521">
+        <v>2520</v>
+      </c>
+      <c r="B2521" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="C2521" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2522" spans="1:3">
+      <c r="A2522">
+        <v>2521</v>
+      </c>
+      <c r="B2522" s="1" t="s">
+        <v>2552</v>
+      </c>
+      <c r="C2522" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2523" spans="1:3">
+      <c r="A2523">
+        <v>2522</v>
+      </c>
+      <c r="B2523" s="1" t="s">
+        <v>2072</v>
+      </c>
+      <c r="C2523" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2524" spans="1:3">
+      <c r="A2524">
+        <v>2523</v>
+      </c>
+      <c r="B2524" s="1" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C2524" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2525" spans="1:3">
+      <c r="A2525">
+        <v>2524</v>
+      </c>
+      <c r="B2525" s="1" t="s">
+        <v>2296</v>
+      </c>
+      <c r="C2525" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2526" spans="1:3">
+      <c r="A2526">
+        <v>2525</v>
+      </c>
+      <c r="B2526" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="C2526" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2527" spans="1:3">
+      <c r="A2527">
+        <v>2526</v>
+      </c>
+      <c r="B2527" s="1" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C2527" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2528" spans="1:3">
+      <c r="A2528">
+        <v>2527</v>
+      </c>
+      <c r="B2528" s="1" t="s">
+        <v>1857</v>
+      </c>
+      <c r="C2528" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2529" spans="1:3">
+      <c r="A2529">
+        <v>2528</v>
+      </c>
+      <c r="B2529" s="1" t="s">
+        <v>2551</v>
+      </c>
+      <c r="C2529" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2530" spans="1:3">
+      <c r="A2530">
+        <v>2529</v>
+      </c>
+      <c r="B2530" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2530" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2531" spans="1:3">
+      <c r="A2531">
+        <v>2530</v>
+      </c>
+      <c r="B2531" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2531" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2532" spans="1:3">
+      <c r="A2532">
+        <v>2531</v>
+      </c>
+      <c r="B2532" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="C2532" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2533" spans="1:3">
+      <c r="A2533">
+        <v>2532</v>
+      </c>
+      <c r="B2533" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="C2533" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2534" spans="1:3">
+      <c r="A2534">
+        <v>2533</v>
+      </c>
+      <c r="B2534" s="1" t="s">
+        <v>2553</v>
+      </c>
+      <c r="C2534" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2535" spans="1:3">
+      <c r="A2535">
+        <v>2534</v>
+      </c>
+      <c r="B2535" s="1" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C2535" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2536" spans="1:3">
+      <c r="A2536">
+        <v>2535</v>
+      </c>
+      <c r="B2536" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C2536" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2537" spans="1:3">
+      <c r="A2537">
+        <v>2536</v>
+      </c>
+      <c r="B2537" s="1" t="s">
+        <v>1957</v>
+      </c>
+      <c r="C2537" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2538" spans="1:3">
+      <c r="A2538">
+        <v>2537</v>
+      </c>
+      <c r="B2538" s="1" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C2538" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2539" spans="1:3">
+      <c r="A2539">
+        <v>2538</v>
+      </c>
+      <c r="B2539" s="1" t="s">
+        <v>2336</v>
+      </c>
+      <c r="C2539" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2540" spans="1:3">
+      <c r="A2540">
+        <v>2539</v>
+      </c>
+      <c r="B2540" s="1" t="s">
+        <v>2497</v>
+      </c>
+      <c r="C2540" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2541" spans="1:3">
+      <c r="A2541">
+        <v>2540</v>
+      </c>
+      <c r="B2541" s="1" t="s">
+        <v>2134</v>
+      </c>
+      <c r="C2541" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2542" spans="1:3">
+      <c r="A2542">
+        <v>2541</v>
+      </c>
+      <c r="B2542" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2542" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2543" spans="1:3">
+      <c r="A2543">
+        <v>2542</v>
+      </c>
+      <c r="B2543" s="1" t="s">
+        <v>1261</v>
+      </c>
+      <c r="C2543" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2544" spans="1:3">
+      <c r="A2544">
+        <v>2543</v>
+      </c>
+      <c r="B2544" s="1" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C2544" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2545" spans="1:3">
+      <c r="A2545">
+        <v>2544</v>
+      </c>
+      <c r="B2545" s="1" t="s">
+        <v>2554</v>
+      </c>
+      <c r="C2545" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2546" spans="1:3">
+      <c r="A2546">
+        <v>2545</v>
+      </c>
+      <c r="B2546" s="1" t="s">
+        <v>1915</v>
+      </c>
+      <c r="C2546" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2547" spans="1:3">
+      <c r="A2547">
+        <v>2546</v>
+      </c>
+      <c r="B2547" s="1" t="s">
+        <v>2186</v>
+      </c>
+      <c r="C2547" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2548" spans="1:3">
+      <c r="A2548">
+        <v>2547</v>
+      </c>
+      <c r="B2548" s="1" t="s">
+        <v>1831</v>
+      </c>
+      <c r="C2548" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2549" spans="1:3">
+      <c r="A2549">
+        <v>2548</v>
+      </c>
+      <c r="B2549" s="1" t="s">
+        <v>2465</v>
+      </c>
+      <c r="C2549" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2550" spans="1:3">
+      <c r="A2550">
+        <v>2549</v>
+      </c>
+      <c r="B2550" s="1" t="s">
+        <v>2434</v>
+      </c>
+      <c r="C2550" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2551" spans="1:3">
+      <c r="A2551">
+        <v>2550</v>
+      </c>
+      <c r="B2551" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="C2551" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2552" spans="1:3">
+      <c r="A2552">
+        <v>2551</v>
+      </c>
+      <c r="B2552" s="1" t="s">
+        <v>2398</v>
+      </c>
+      <c r="C2552" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2553" spans="1:3">
+      <c r="A2553">
+        <v>2552</v>
+      </c>
+      <c r="B2553" s="1" t="s">
+        <v>2351</v>
+      </c>
+      <c r="C2553" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2554" spans="1:3">
+      <c r="A2554">
+        <v>2553</v>
+      </c>
+      <c r="B2554" s="1" t="s">
+        <v>2550</v>
+      </c>
+      <c r="C2554" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2555" spans="1:3">
+      <c r="A2555">
+        <v>2554</v>
+      </c>
+      <c r="B2555" s="1" t="s">
+        <v>1305</v>
+      </c>
+      <c r="C2555" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2556" spans="1:3">
+      <c r="A2556">
+        <v>2555</v>
+      </c>
+      <c r="B2556" s="1" t="s">
+        <v>2097</v>
+      </c>
+      <c r="C2556" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2557" spans="1:3">
+      <c r="A2557">
+        <v>2556</v>
+      </c>
+      <c r="B2557" s="1" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C2557" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2558" spans="1:3">
+      <c r="A2558">
+        <v>2557</v>
+      </c>
+      <c r="B2558" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="C2558" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2559" spans="1:3">
+      <c r="A2559">
+        <v>2558</v>
+      </c>
+      <c r="B2559" s="1" t="s">
+        <v>1536</v>
+      </c>
+      <c r="C2559" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2560" spans="1:3">
+      <c r="A2560">
+        <v>2559</v>
+      </c>
+      <c r="B2560" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="C2560" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2561" spans="1:3">
+      <c r="A2561">
+        <v>2560</v>
+      </c>
+      <c r="B2561" s="1" t="s">
+        <v>2555</v>
+      </c>
+      <c r="C2561" t="s">
+        <v>2556</v>
+      </c>
+    </row>
+    <row r="2562" spans="1:3">
+      <c r="A2562">
+        <v>2561</v>
+      </c>
+      <c r="B2562" s="1" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C2562" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2563" spans="1:3">
+      <c r="A2563">
+        <v>2562</v>
+      </c>
+      <c r="B2563" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="C2563" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2564" spans="1:3">
+      <c r="A2564">
+        <v>2563</v>
+      </c>
+      <c r="B2564" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="C2564" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2565" spans="1:3">
+      <c r="A2565">
+        <v>2564</v>
+      </c>
+      <c r="B2565" s="1" t="s">
+        <v>885</v>
+      </c>
+      <c r="C2565" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2566" spans="1:3">
+      <c r="A2566">
+        <v>2565</v>
+      </c>
+      <c r="B2566" s="1" t="s">
+        <v>396</v>
+      </c>
+      <c r="C2566" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2567" spans="1:3">
+      <c r="A2567">
+        <v>2566</v>
+      </c>
+      <c r="B2567" s="1" t="s">
+        <v>2025</v>
+      </c>
+      <c r="C2567" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2568" spans="1:3">
+      <c r="A2568">
+        <v>2567</v>
+      </c>
+      <c r="B2568" s="1" t="s">
+        <v>639</v>
+      </c>
+      <c r="C2568" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2569" spans="1:3">
+      <c r="A2569">
+        <v>2568</v>
+      </c>
+      <c r="B2569" s="1" t="s">
+        <v>1474</v>
+      </c>
+      <c r="C2569" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2570" spans="1:3">
+      <c r="A2570">
+        <v>2569</v>
+      </c>
+      <c r="B2570" s="1" t="s">
+        <v>1608</v>
+      </c>
+      <c r="C2570" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2571" spans="1:3">
+      <c r="A2571">
+        <v>2570</v>
+      </c>
+      <c r="B2571" s="1" t="s">
+        <v>965</v>
+      </c>
+      <c r="C2571" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2572" spans="1:3">
+      <c r="A2572">
+        <v>2571</v>
+      </c>
+      <c r="B2572" s="1" t="s">
+        <v>1653</v>
+      </c>
+      <c r="C2572" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2573" spans="1:3">
+      <c r="A2573">
+        <v>2572</v>
+      </c>
+      <c r="B2573" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2573" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2574" spans="1:3">
+      <c r="A2574">
+        <v>2573</v>
+      </c>
+      <c r="B2574" s="1" t="s">
+        <v>546</v>
+      </c>
+      <c r="C2574" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2575" spans="1:3">
+      <c r="A2575">
+        <v>2574</v>
+      </c>
+      <c r="B2575" s="1" t="s">
+        <v>2552</v>
+      </c>
+      <c r="C2575" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2576" spans="1:3">
+      <c r="A2576">
+        <v>2575</v>
+      </c>
+      <c r="B2576" s="1" t="s">
+        <v>2072</v>
+      </c>
+      <c r="C2576" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2577" spans="1:3">
+      <c r="A2577">
+        <v>2576</v>
+      </c>
+      <c r="B2577" s="1" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C2577" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2578" spans="1:3">
+      <c r="A2578">
+        <v>2577</v>
+      </c>
+      <c r="B2578" s="1" t="s">
+        <v>2296</v>
+      </c>
+      <c r="C2578" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2579" spans="1:3">
+      <c r="A2579">
+        <v>2578</v>
+      </c>
+      <c r="B2579" s="1" t="s">
+        <v>689</v>
+      </c>
+      <c r="C2579" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2580" spans="1:3">
+      <c r="A2580">
+        <v>2579</v>
+      </c>
+      <c r="B2580" s="1" t="s">
+        <v>1219</v>
+      </c>
+      <c r="C2580" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2581" spans="1:3">
+      <c r="A2581">
+        <v>2580</v>
+      </c>
+      <c r="B2581" s="1" t="s">
+        <v>1857</v>
+      </c>
+      <c r="C2581" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2582" spans="1:3">
+      <c r="A2582">
+        <v>2581</v>
+      </c>
+      <c r="B2582" s="1" t="s">
+        <v>2551</v>
+      </c>
+      <c r="C2582" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2583" spans="1:3">
+      <c r="A2583">
+        <v>2582</v>
+      </c>
+      <c r="B2583" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2583" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2584" spans="1:3">
+      <c r="A2584">
+        <v>2583</v>
+      </c>
+      <c r="B2584" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2584" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2585" spans="1:3">
+      <c r="A2585">
+        <v>2584</v>
+      </c>
+      <c r="B2585" s="1" t="s">
+        <v>843</v>
+      </c>
+      <c r="C2585" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2586" spans="1:3">
+      <c r="A2586">
+        <v>2585</v>
+      </c>
+      <c r="B2586" s="1" t="s">
+        <v>732</v>
+      </c>
+      <c r="C2586" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2587" spans="1:3">
+      <c r="A2587">
+        <v>2586</v>
+      </c>
+      <c r="B2587" s="1" t="s">
+        <v>2553</v>
+      </c>
+      <c r="C2587" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2588" spans="1:3">
+      <c r="A2588">
+        <v>2587</v>
+      </c>
+      <c r="B2588" s="1" t="s">
+        <v>1729</v>
+      </c>
+      <c r="C2588" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2589" spans="1:3">
+      <c r="A2589">
+        <v>2588</v>
+      </c>
+      <c r="B2589" s="1" t="s">
+        <v>596</v>
+      </c>
+      <c r="C2589" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2590" spans="1:3">
+      <c r="A2590">
+        <v>2589</v>
+      </c>
+      <c r="B2590" s="1" t="s">
+        <v>1957</v>
+      </c>
+      <c r="C2590" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2591" spans="1:3">
+      <c r="A2591">
+        <v>2590</v>
+      </c>
+      <c r="B2591" s="1" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C2591" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2592" spans="1:3">
+      <c r="A2592">
+        <v>2591</v>
+      </c>
+      <c r="B2592" s="1" t="s">
+        <v>2336</v>
+      </c>
+      <c r="C2592" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2593" spans="1:3">
+      <c r="A2593">
+        <v>2592</v>
+      </c>
+      <c r="B2593" s="1" t="s">
+        <v>2497</v>
+      </c>
+      <c r="C2593" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2594" spans="1:3">
+      <c r="A2594">
+        <v>2593</v>
+      </c>
+      <c r="B2594" s="1" t="s">
+        <v>2134</v>
+      </c>
+      <c r="C2594" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2595" spans="1:3">
+      <c r="A2595">
+        <v>2594</v>
+      </c>
+      <c r="B2595" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2595" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2596" spans="1:3">
+      <c r="A2596">
+        <v>2595</v>
+      </c>
+      <c r="B2596" s="1" t="s">
+        <v>1261</v>
+      </c>
+      <c r="C2596" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2597" spans="1:3">
+      <c r="A2597">
+        <v>2596</v>
+      </c>
+      <c r="B2597" s="1" t="s">
+        <v>1011</v>
+      </c>
+      <c r="C2597" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2598" spans="1:3">
+      <c r="A2598">
+        <v>2597</v>
+      </c>
+      <c r="B2598" s="1" t="s">
+        <v>2554</v>
+      </c>
+      <c r="C2598" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2599" spans="1:3">
+      <c r="A2599">
+        <v>2598</v>
+      </c>
+      <c r="B2599" s="1" t="s">
+        <v>1915</v>
+      </c>
+      <c r="C2599" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2600" spans="1:3">
+      <c r="A2600">
+        <v>2599</v>
+      </c>
+      <c r="B2600" s="1" t="s">
+        <v>2186</v>
+      </c>
+      <c r="C2600" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2601" spans="1:3">
+      <c r="A2601">
+        <v>2600</v>
+      </c>
+      <c r="B2601" s="1" t="s">
+        <v>1831</v>
+      </c>
+      <c r="C2601" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2602" spans="1:3">
+      <c r="A2602">
+        <v>2601</v>
+      </c>
+      <c r="B2602" s="1" t="s">
+        <v>2465</v>
+      </c>
+      <c r="C2602" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2603" spans="1:3">
+      <c r="A2603">
+        <v>2602</v>
+      </c>
+      <c r="B2603" s="1" t="s">
+        <v>2434</v>
+      </c>
+      <c r="C2603" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2604" spans="1:3">
+      <c r="A2604">
+        <v>2603</v>
+      </c>
+      <c r="B2604" s="1" t="s">
+        <v>505</v>
+      </c>
+      <c r="C2604" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2605" spans="1:3">
+      <c r="A2605">
+        <v>2604</v>
+      </c>
+      <c r="B2605" s="1" t="s">
+        <v>2398</v>
+      </c>
+      <c r="C2605" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2606" spans="1:3">
+      <c r="A2606">
+        <v>2605</v>
+      </c>
+      <c r="B2606" s="1" t="s">
+        <v>2351</v>
+      </c>
+      <c r="C2606" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2607" spans="1:3">
+      <c r="A2607">
+        <v>2606</v>
+      </c>
+      <c r="B2607" s="1" t="s">
+        <v>2550</v>
+      </c>
+      <c r="C2607" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2608" spans="1:3">
+      <c r="A2608">
+        <v>2607</v>
+      </c>
+      <c r="B2608" s="1" t="s">
+        <v>1305</v>
+      </c>
+      <c r="C2608" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2609" spans="1:3">
+      <c r="A2609">
+        <v>2608</v>
+      </c>
+      <c r="B2609" s="1" t="s">
+        <v>2097</v>
+      </c>
+      <c r="C2609" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2610" spans="1:3">
+      <c r="A2610">
+        <v>2609</v>
+      </c>
+      <c r="B2610" s="1" t="s">
+        <v>1287</v>
+      </c>
+      <c r="C2610" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2611" spans="1:3">
+      <c r="A2611">
+        <v>2610</v>
+      </c>
+      <c r="B2611" s="1" t="s">
+        <v>443</v>
+      </c>
+      <c r="C2611" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2612" spans="1:3">
+      <c r="A2612">
+        <v>2611</v>
+      </c>
+      <c r="B2612" s="1" t="s">
+        <v>1536</v>
+      </c>
+      <c r="C2612" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2613" spans="1:3">
+      <c r="A2613">
+        <v>2612</v>
+      </c>
+      <c r="B2613" s="1" t="s">
+        <v>771</v>
+      </c>
+      <c r="C2613" t="s">
+        <v>2557</v>
+      </c>
+    </row>
+    <row r="2614" spans="1:3">
+      <c r="A2614">
+        <v>2613</v>
+      </c>
+      <c r="B2614" s="1" t="s">
+        <v>2555</v>
+      </c>
+      <c r="C2614" t="s">
+        <v>2557</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
s.no., na, bolero, total, local repair
</commit_message>
<xml_diff>
--- a/VEHAPR26.xlsx
+++ b/VEHAPR26.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5229" uniqueCount="2558">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5335" uniqueCount="2559">
   <si>
     <t>NAME</t>
   </si>
@@ -7691,6 +7691,9 @@
   </si>
   <si>
     <t>RJ37PA2306</t>
+  </si>
+  <si>
+    <t>BOLERO</t>
   </si>
 </sst>
 </file>
@@ -8025,7 +8028,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2614"/>
+  <dimension ref="A1:C2667"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -36812,6 +36815,589 @@
         <v>2551</v>
       </c>
     </row>
+    <row r="2615" spans="1:3">
+      <c r="A2615">
+        <v>2614</v>
+      </c>
+      <c r="B2615" s="1" t="s">
+        <v>2162</v>
+      </c>
+      <c r="C2615" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2616" spans="1:3">
+      <c r="A2616">
+        <v>2615</v>
+      </c>
+      <c r="B2616" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C2616" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2617" spans="1:3">
+      <c r="A2617">
+        <v>2616</v>
+      </c>
+      <c r="B2617" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C2617" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2618" spans="1:3">
+      <c r="A2618">
+        <v>2617</v>
+      </c>
+      <c r="B2618" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="C2618" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2619" spans="1:3">
+      <c r="A2619">
+        <v>2618</v>
+      </c>
+      <c r="B2619" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="C2619" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2620" spans="1:3">
+      <c r="A2620">
+        <v>2619</v>
+      </c>
+      <c r="B2620" s="1" t="s">
+        <v>2018</v>
+      </c>
+      <c r="C2620" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2621" spans="1:3">
+      <c r="A2621">
+        <v>2620</v>
+      </c>
+      <c r="B2621" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="C2621" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2622" spans="1:3">
+      <c r="A2622">
+        <v>2621</v>
+      </c>
+      <c r="B2622" s="1" t="s">
+        <v>1472</v>
+      </c>
+      <c r="C2622" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2623" spans="1:3">
+      <c r="A2623">
+        <v>2622</v>
+      </c>
+      <c r="B2623" s="1" t="s">
+        <v>1606</v>
+      </c>
+      <c r="C2623" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2624" spans="1:3">
+      <c r="A2624">
+        <v>2623</v>
+      </c>
+      <c r="B2624" s="1" t="s">
+        <v>963</v>
+      </c>
+      <c r="C2624" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2625" spans="1:3">
+      <c r="A2625">
+        <v>2624</v>
+      </c>
+      <c r="B2625" s="1" t="s">
+        <v>1649</v>
+      </c>
+      <c r="C2625" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2626" spans="1:3">
+      <c r="A2626">
+        <v>2625</v>
+      </c>
+      <c r="B2626" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2626" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2627" spans="1:3">
+      <c r="A2627">
+        <v>2626</v>
+      </c>
+      <c r="B2627" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="C2627" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2628" spans="1:3">
+      <c r="A2628">
+        <v>2627</v>
+      </c>
+      <c r="B2628" s="1" t="s">
+        <v>2544</v>
+      </c>
+      <c r="C2628" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2629" spans="1:3">
+      <c r="A2629">
+        <v>2628</v>
+      </c>
+      <c r="B2629" s="1" t="s">
+        <v>2065</v>
+      </c>
+      <c r="C2629" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2630" spans="1:3">
+      <c r="A2630">
+        <v>2629</v>
+      </c>
+      <c r="B2630" s="1" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C2630" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2631" spans="1:3">
+      <c r="A2631">
+        <v>2630</v>
+      </c>
+      <c r="B2631" s="1" t="s">
+        <v>2289</v>
+      </c>
+      <c r="C2631" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2632" spans="1:3">
+      <c r="A2632">
+        <v>2631</v>
+      </c>
+      <c r="B2632" s="1" t="s">
+        <v>687</v>
+      </c>
+      <c r="C2632" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2633" spans="1:3">
+      <c r="A2633">
+        <v>2632</v>
+      </c>
+      <c r="B2633" s="1" t="s">
+        <v>1217</v>
+      </c>
+      <c r="C2633" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2634" spans="1:3">
+      <c r="A2634">
+        <v>2633</v>
+      </c>
+      <c r="B2634" s="1" t="s">
+        <v>1850</v>
+      </c>
+      <c r="C2634" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2635" spans="1:3">
+      <c r="A2635">
+        <v>2634</v>
+      </c>
+      <c r="B2635" s="1" t="s">
+        <v>2543</v>
+      </c>
+      <c r="C2635" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2636" spans="1:3">
+      <c r="A2636">
+        <v>2635</v>
+      </c>
+      <c r="B2636" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2636" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2637" spans="1:3">
+      <c r="A2637">
+        <v>2636</v>
+      </c>
+      <c r="B2637" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2637" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2638" spans="1:3">
+      <c r="A2638">
+        <v>2637</v>
+      </c>
+      <c r="B2638" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="C2638" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2639" spans="1:3">
+      <c r="A2639">
+        <v>2638</v>
+      </c>
+      <c r="B2639" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="C2639" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2640" spans="1:3">
+      <c r="A2640">
+        <v>2639</v>
+      </c>
+      <c r="B2640" s="1" t="s">
+        <v>2545</v>
+      </c>
+      <c r="C2640" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2641" spans="1:3">
+      <c r="A2641">
+        <v>2640</v>
+      </c>
+      <c r="B2641" s="1" t="s">
+        <v>1725</v>
+      </c>
+      <c r="C2641" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2642" spans="1:3">
+      <c r="A2642">
+        <v>2641</v>
+      </c>
+      <c r="B2642" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="C2642" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2643" spans="1:3">
+      <c r="A2643">
+        <v>2642</v>
+      </c>
+      <c r="B2643" s="1" t="s">
+        <v>1950</v>
+      </c>
+      <c r="C2643" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2644" spans="1:3">
+      <c r="A2644">
+        <v>2643</v>
+      </c>
+      <c r="B2644" s="1" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C2644" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2645" spans="1:3">
+      <c r="A2645">
+        <v>2644</v>
+      </c>
+      <c r="B2645" s="1" t="s">
+        <v>2328</v>
+      </c>
+      <c r="C2645" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2646" spans="1:3">
+      <c r="A2646">
+        <v>2645</v>
+      </c>
+      <c r="B2646" s="1" t="s">
+        <v>2489</v>
+      </c>
+      <c r="C2646" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2647" spans="1:3">
+      <c r="A2647">
+        <v>2646</v>
+      </c>
+      <c r="B2647" s="1" t="s">
+        <v>2127</v>
+      </c>
+      <c r="C2647" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2648" spans="1:3">
+      <c r="A2648">
+        <v>2647</v>
+      </c>
+      <c r="B2648" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2648" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2649" spans="1:3">
+      <c r="A2649">
+        <v>2648</v>
+      </c>
+      <c r="B2649" s="1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="C2649" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2650" spans="1:3">
+      <c r="A2650">
+        <v>2649</v>
+      </c>
+      <c r="B2650" s="1" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C2650" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2651" spans="1:3">
+      <c r="A2651">
+        <v>2650</v>
+      </c>
+      <c r="B2651" s="1" t="s">
+        <v>2546</v>
+      </c>
+      <c r="C2651" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2652" spans="1:3">
+      <c r="A2652">
+        <v>2651</v>
+      </c>
+      <c r="B2652" s="1" t="s">
+        <v>1908</v>
+      </c>
+      <c r="C2652" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2653" spans="1:3">
+      <c r="A2653">
+        <v>2652</v>
+      </c>
+      <c r="B2653" s="1" t="s">
+        <v>2179</v>
+      </c>
+      <c r="C2653" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2654" spans="1:3">
+      <c r="A2654">
+        <v>2653</v>
+      </c>
+      <c r="B2654" s="1" t="s">
+        <v>1824</v>
+      </c>
+      <c r="C2654" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2655" spans="1:3">
+      <c r="A2655">
+        <v>2654</v>
+      </c>
+      <c r="B2655" s="1" t="s">
+        <v>2457</v>
+      </c>
+      <c r="C2655" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2656" spans="1:3">
+      <c r="A2656">
+        <v>2655</v>
+      </c>
+      <c r="B2656" s="1" t="s">
+        <v>2426</v>
+      </c>
+      <c r="C2656" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2657" spans="1:3">
+      <c r="A2657">
+        <v>2656</v>
+      </c>
+      <c r="B2657" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="C2657" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2658" spans="1:3">
+      <c r="A2658">
+        <v>2657</v>
+      </c>
+      <c r="B2658" s="1" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C2658" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2659" spans="1:3">
+      <c r="A2659">
+        <v>2658</v>
+      </c>
+      <c r="B2659" s="1" t="s">
+        <v>2343</v>
+      </c>
+      <c r="C2659" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2660" spans="1:3">
+      <c r="A2660">
+        <v>2659</v>
+      </c>
+      <c r="B2660" s="1" t="s">
+        <v>2542</v>
+      </c>
+      <c r="C2660" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2661" spans="1:3">
+      <c r="A2661">
+        <v>2660</v>
+      </c>
+      <c r="B2661" s="1" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C2661" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2662" spans="1:3">
+      <c r="A2662">
+        <v>2661</v>
+      </c>
+      <c r="B2662" s="1" t="s">
+        <v>2090</v>
+      </c>
+      <c r="C2662" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2663" spans="1:3">
+      <c r="A2663">
+        <v>2662</v>
+      </c>
+      <c r="B2663" s="1" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C2663" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2664" spans="1:3">
+      <c r="A2664">
+        <v>2663</v>
+      </c>
+      <c r="B2664" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="C2664" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2665" spans="1:3">
+      <c r="A2665">
+        <v>2664</v>
+      </c>
+      <c r="B2665" s="1" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C2665" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2666" spans="1:3">
+      <c r="A2666">
+        <v>2665</v>
+      </c>
+      <c r="B2666" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="C2666" t="s">
+        <v>2558</v>
+      </c>
+    </row>
+    <row r="2667" spans="1:3">
+      <c r="A2667">
+        <v>2666</v>
+      </c>
+      <c r="B2667" s="1" t="s">
+        <v>2547</v>
+      </c>
+      <c r="C2667" t="s">
+        <v>2558</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Updated RSRTC Indent System
</commit_message>
<xml_diff>
--- a/VEHAPR26.xlsx
+++ b/VEHAPR26.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5335" uniqueCount="2559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5441" uniqueCount="2560">
   <si>
     <t>NAME</t>
   </si>
@@ -7694,6 +7694,9 @@
   </si>
   <si>
     <t>BOLERO</t>
+  </si>
+  <si>
+    <t>TRUCK</t>
   </si>
 </sst>
 </file>
@@ -8028,7 +8031,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2667"/>
+  <dimension ref="A1:C2720"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -37398,6 +37401,589 @@
         <v>2558</v>
       </c>
     </row>
+    <row r="2668" spans="1:3">
+      <c r="A2668">
+        <v>2667</v>
+      </c>
+      <c r="B2668" s="1" t="s">
+        <v>2162</v>
+      </c>
+      <c r="C2668" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2669" spans="1:3">
+      <c r="A2669">
+        <v>2668</v>
+      </c>
+      <c r="B2669" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="C2669" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2670" spans="1:3">
+      <c r="A2670">
+        <v>2669</v>
+      </c>
+      <c r="B2670" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C2670" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2671" spans="1:3">
+      <c r="A2671">
+        <v>2670</v>
+      </c>
+      <c r="B2671" s="1" t="s">
+        <v>883</v>
+      </c>
+      <c r="C2671" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2672" spans="1:3">
+      <c r="A2672">
+        <v>2671</v>
+      </c>
+      <c r="B2672" s="1" t="s">
+        <v>394</v>
+      </c>
+      <c r="C2672" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2673" spans="1:3">
+      <c r="A2673">
+        <v>2672</v>
+      </c>
+      <c r="B2673" s="1" t="s">
+        <v>2018</v>
+      </c>
+      <c r="C2673" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2674" spans="1:3">
+      <c r="A2674">
+        <v>2673</v>
+      </c>
+      <c r="B2674" s="1" t="s">
+        <v>637</v>
+      </c>
+      <c r="C2674" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2675" spans="1:3">
+      <c r="A2675">
+        <v>2674</v>
+      </c>
+      <c r="B2675" s="1" t="s">
+        <v>1472</v>
+      </c>
+      <c r="C2675" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2676" spans="1:3">
+      <c r="A2676">
+        <v>2675</v>
+      </c>
+      <c r="B2676" s="1" t="s">
+        <v>1606</v>
+      </c>
+      <c r="C2676" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2677" spans="1:3">
+      <c r="A2677">
+        <v>2676</v>
+      </c>
+      <c r="B2677" s="1" t="s">
+        <v>963</v>
+      </c>
+      <c r="C2677" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2678" spans="1:3">
+      <c r="A2678">
+        <v>2677</v>
+      </c>
+      <c r="B2678" s="1" t="s">
+        <v>1649</v>
+      </c>
+      <c r="C2678" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2679" spans="1:3">
+      <c r="A2679">
+        <v>2678</v>
+      </c>
+      <c r="B2679" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2679" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2680" spans="1:3">
+      <c r="A2680">
+        <v>2679</v>
+      </c>
+      <c r="B2680" s="1" t="s">
+        <v>544</v>
+      </c>
+      <c r="C2680" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2681" spans="1:3">
+      <c r="A2681">
+        <v>2680</v>
+      </c>
+      <c r="B2681" s="1" t="s">
+        <v>2544</v>
+      </c>
+      <c r="C2681" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2682" spans="1:3">
+      <c r="A2682">
+        <v>2681</v>
+      </c>
+      <c r="B2682" s="1" t="s">
+        <v>2065</v>
+      </c>
+      <c r="C2682" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2683" spans="1:3">
+      <c r="A2683">
+        <v>2682</v>
+      </c>
+      <c r="B2683" s="1" t="s">
+        <v>1102</v>
+      </c>
+      <c r="C2683" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2684" spans="1:3">
+      <c r="A2684">
+        <v>2683</v>
+      </c>
+      <c r="B2684" s="1" t="s">
+        <v>2289</v>
+      </c>
+      <c r="C2684" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2685" spans="1:3">
+      <c r="A2685">
+        <v>2684</v>
+      </c>
+      <c r="B2685" s="1" t="s">
+        <v>687</v>
+      </c>
+      <c r="C2685" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2686" spans="1:3">
+      <c r="A2686">
+        <v>2685</v>
+      </c>
+      <c r="B2686" s="1" t="s">
+        <v>1217</v>
+      </c>
+      <c r="C2686" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2687" spans="1:3">
+      <c r="A2687">
+        <v>2686</v>
+      </c>
+      <c r="B2687" s="1" t="s">
+        <v>1850</v>
+      </c>
+      <c r="C2687" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2688" spans="1:3">
+      <c r="A2688">
+        <v>2687</v>
+      </c>
+      <c r="B2688" s="1" t="s">
+        <v>2543</v>
+      </c>
+      <c r="C2688" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2689" spans="1:3">
+      <c r="A2689">
+        <v>2688</v>
+      </c>
+      <c r="B2689" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2689" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2690" spans="1:3">
+      <c r="A2690">
+        <v>2689</v>
+      </c>
+      <c r="B2690" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C2690" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2691" spans="1:3">
+      <c r="A2691">
+        <v>2690</v>
+      </c>
+      <c r="B2691" s="1" t="s">
+        <v>841</v>
+      </c>
+      <c r="C2691" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2692" spans="1:3">
+      <c r="A2692">
+        <v>2691</v>
+      </c>
+      <c r="B2692" s="1" t="s">
+        <v>730</v>
+      </c>
+      <c r="C2692" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2693" spans="1:3">
+      <c r="A2693">
+        <v>2692</v>
+      </c>
+      <c r="B2693" s="1" t="s">
+        <v>2545</v>
+      </c>
+      <c r="C2693" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2694" spans="1:3">
+      <c r="A2694">
+        <v>2693</v>
+      </c>
+      <c r="B2694" s="1" t="s">
+        <v>1725</v>
+      </c>
+      <c r="C2694" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2695" spans="1:3">
+      <c r="A2695">
+        <v>2694</v>
+      </c>
+      <c r="B2695" s="1" t="s">
+        <v>594</v>
+      </c>
+      <c r="C2695" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2696" spans="1:3">
+      <c r="A2696">
+        <v>2695</v>
+      </c>
+      <c r="B2696" s="1" t="s">
+        <v>1950</v>
+      </c>
+      <c r="C2696" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2697" spans="1:3">
+      <c r="A2697">
+        <v>2696</v>
+      </c>
+      <c r="B2697" s="1" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C2697" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2698" spans="1:3">
+      <c r="A2698">
+        <v>2697</v>
+      </c>
+      <c r="B2698" s="1" t="s">
+        <v>2328</v>
+      </c>
+      <c r="C2698" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2699" spans="1:3">
+      <c r="A2699">
+        <v>2698</v>
+      </c>
+      <c r="B2699" s="1" t="s">
+        <v>2489</v>
+      </c>
+      <c r="C2699" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2700" spans="1:3">
+      <c r="A2700">
+        <v>2699</v>
+      </c>
+      <c r="B2700" s="1" t="s">
+        <v>2127</v>
+      </c>
+      <c r="C2700" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2701" spans="1:3">
+      <c r="A2701">
+        <v>2700</v>
+      </c>
+      <c r="B2701" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2701" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2702" spans="1:3">
+      <c r="A2702">
+        <v>2701</v>
+      </c>
+      <c r="B2702" s="1" t="s">
+        <v>1259</v>
+      </c>
+      <c r="C2702" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2703" spans="1:3">
+      <c r="A2703">
+        <v>2702</v>
+      </c>
+      <c r="B2703" s="1" t="s">
+        <v>1009</v>
+      </c>
+      <c r="C2703" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2704" spans="1:3">
+      <c r="A2704">
+        <v>2703</v>
+      </c>
+      <c r="B2704" s="1" t="s">
+        <v>2546</v>
+      </c>
+      <c r="C2704" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2705" spans="1:3">
+      <c r="A2705">
+        <v>2704</v>
+      </c>
+      <c r="B2705" s="1" t="s">
+        <v>1908</v>
+      </c>
+      <c r="C2705" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2706" spans="1:3">
+      <c r="A2706">
+        <v>2705</v>
+      </c>
+      <c r="B2706" s="1" t="s">
+        <v>2179</v>
+      </c>
+      <c r="C2706" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2707" spans="1:3">
+      <c r="A2707">
+        <v>2706</v>
+      </c>
+      <c r="B2707" s="1" t="s">
+        <v>1824</v>
+      </c>
+      <c r="C2707" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2708" spans="1:3">
+      <c r="A2708">
+        <v>2707</v>
+      </c>
+      <c r="B2708" s="1" t="s">
+        <v>2457</v>
+      </c>
+      <c r="C2708" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2709" spans="1:3">
+      <c r="A2709">
+        <v>2708</v>
+      </c>
+      <c r="B2709" s="1" t="s">
+        <v>2426</v>
+      </c>
+      <c r="C2709" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2710" spans="1:3">
+      <c r="A2710">
+        <v>2709</v>
+      </c>
+      <c r="B2710" s="1" t="s">
+        <v>503</v>
+      </c>
+      <c r="C2710" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2711" spans="1:3">
+      <c r="A2711">
+        <v>2710</v>
+      </c>
+      <c r="B2711" s="1" t="s">
+        <v>2390</v>
+      </c>
+      <c r="C2711" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2712" spans="1:3">
+      <c r="A2712">
+        <v>2711</v>
+      </c>
+      <c r="B2712" s="1" t="s">
+        <v>2343</v>
+      </c>
+      <c r="C2712" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2713" spans="1:3">
+      <c r="A2713">
+        <v>2712</v>
+      </c>
+      <c r="B2713" s="1" t="s">
+        <v>2542</v>
+      </c>
+      <c r="C2713" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2714" spans="1:3">
+      <c r="A2714">
+        <v>2713</v>
+      </c>
+      <c r="B2714" s="1" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C2714" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2715" spans="1:3">
+      <c r="A2715">
+        <v>2714</v>
+      </c>
+      <c r="B2715" s="1" t="s">
+        <v>2090</v>
+      </c>
+      <c r="C2715" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2716" spans="1:3">
+      <c r="A2716">
+        <v>2715</v>
+      </c>
+      <c r="B2716" s="1" t="s">
+        <v>1285</v>
+      </c>
+      <c r="C2716" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2717" spans="1:3">
+      <c r="A2717">
+        <v>2716</v>
+      </c>
+      <c r="B2717" s="1" t="s">
+        <v>441</v>
+      </c>
+      <c r="C2717" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2718" spans="1:3">
+      <c r="A2718">
+        <v>2717</v>
+      </c>
+      <c r="B2718" s="1" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C2718" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2719" spans="1:3">
+      <c r="A2719">
+        <v>2718</v>
+      </c>
+      <c r="B2719" s="1" t="s">
+        <v>769</v>
+      </c>
+      <c r="C2719" t="s">
+        <v>2559</v>
+      </c>
+    </row>
+    <row r="2720" spans="1:3">
+      <c r="A2720">
+        <v>2719</v>
+      </c>
+      <c r="B2720" s="1" t="s">
+        <v>2547</v>
+      </c>
+      <c r="C2720" t="s">
+        <v>2559</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:C1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>